<commit_message>
119 Use Cases - Backup wiederhergestellt + 2 neue Vertriebs-Use-Cases
</commit_message>
<xml_diff>
--- a/KI_UseCases_Uebersicht.xlsx
+++ b/KI_UseCases_Uebersicht.xlsx
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Newsletter sind ressourcenintensiv – Themenrecherche, Strukturierung, Layout, Personalisierung pro Zielgruppe, Übersetzung und Versandsteuerung erfordern viele manuelle Schritte; datengetriebene Entscheidungen zu Inhalten und Versandzeitpunkt fehlen, sodass Öffnungs- und Klickraten unter dem Möglichen bleiben</t>
+          <t>Newslettererstellung und -optimierung ist ressourcenintensiv und wenig datengetrieben</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Aufgaben werden vergessen und Fristen verpasst, weil klassische Reminder pauschal sind und den individuellen Arbeitskontext (Aufgabenpriorität, Tagesablauf, bisherige Erledigungsmuster) nicht berücksichtigen – wichtige To-Dos gehen im Tagesgeschäft unter</t>
+          <t>Aufgaben werden vergessen und Fristen verpasst mangels intelligenter, nutzerorientierter Erinnerungen</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Smart Nudging: KI analysiert individuelle To-Do-Muster und Erledigungszeiten, identifiziert die richtigen Momente für eine Erinnerung und setzt kontextbezogene, personalisierte Reminder statt pauschaler Benachrichtigungen</t>
+          <t>Smart Nudging: KI erkennt To-Do-Muster und setzt kontextbasierte Reminder</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">

</xml_diff>